<commit_message>
Update frontend API URL to production
</commit_message>
<xml_diff>
--- a/backend/income_details.xlsx
+++ b/backend/income_details.xlsx
@@ -415,13 +415,13 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>salary</v>
+        <v>w</v>
       </c>
       <c r="B2">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="C2" t="str">
-        <v>Salary</v>
+        <v>Food</v>
       </c>
       <c r="D2" t="str">
         <v>30/6/2026</v>

</xml_diff>